<commit_message>
Restate VRE BVPS and P/B on our own earnings and the cash dividend
P/E was already forward-consistent at every revision. VRE P/B was not:
BVPS came from the VRE model's BS, which (i) embeds FY26/27 net income
of 5,913/6,170 rather than our 5,483/6,305, (ii) returns #DIV/0! in the
forecast columns of its equity roll-forward (Equity!L16/M16), and
(iii) assumes zero dividends despite VRE's first cash payout in 7 years
(~VND2.3tn, Jul-2026).

Rebuilt from FY25 BVPS 20,196 plus our NPATMI less the dividend:
BVPS 21,563 (FY26F) / 23,283 (FY27F), lifting P/B from 1.23x/1.10x to
1.30x/1.20x. Valuation cell and the internal provenance record updated;
the no-FY27-dividend alternative (P/B 1.15x) is documented there.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
+++ b/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1519,12 +1519,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>BVPS / P-B basis</t>
+          <t>BVPS / P-B basis — RESTATED</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>22,798 / 25,513</t>
+          <t>21,563 / 23,283</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -1534,17 +1534,17 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>MODEL</t>
+          <t>MAS</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>VRE model BS!L136 / M136</t>
+          <t>Rebuilt from FY25 BVPS 20,196 (VRE model BS!K136) + our NPATMI less the ~VND2.3tn cash dividend</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr">
         <is>
-          <t>Model balance sheet embeds LOWER earnings than the Stock Pick overrides, so P/B is modestly overstated (~4%).</t>
+          <t>Model BS!L136/M136 (22,798/25,513) NOT used: it embeds FY26/27 NI of 5,913/6,170 rather than our 5,483/6,305, its equity roll-forward returns #DIV/0! in the forecast columns (Equity!L16/M16), and it assumes ZERO dividends despite the first cash payout in 7 years (~VND2.3tn, Jul-2026). Restating lifts P/B from 1.23x/1.10x to 1.30x/1.20x. FY27 assumes the dividend repeats; if not, BVPS27 = 24,270 and P/B27 = 1.15x.</t>
         </is>
       </c>
     </row>
@@ -1771,6 +1771,21 @@
         </is>
       </c>
     </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A3:G3"/>

</xml_diff>

<commit_message>
Plain-language rewrite; remove competitor references; cut VRE text ~20%
1) Jargon removed across the FPT and VRE narrative cells: "property leg
   haircut", "annualise", "lease-up", "optionality", "base-case engine",
   "step-up", "lumpy", "150bp of margin dilution", "flattered",
   "underpins", "insulated from", "GM". Replaced with plain wording.
2) All references to other securities firms removed from the
   client-facing stock pick and the STB/EIB deck; the internal
   provenance file now cites "a competing broker" without naming it.
3) VRE Growth cell cut a further ~18% (1,324 -> 1,089 chars).
4) Fixed a stale figure in the VRE valuation cell: P/B and BVPS now show
   the restated 1.30x / ~VND21,600 rather than the superseded
   1.23x / ~VND22,800.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
+++ b/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -508,6 +508,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -1271,7 +1272,7 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>+20.0%. MBS forecasts 6,502 (+19.2%) on a similar view.</t>
+          <t>+20.0%. a competing broker forecasts 6,502 (+19.2%) on a similar view.</t>
         </is>
       </c>
     </row>
@@ -1771,21 +1772,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A3:G3"/>

</xml_diff>

<commit_message>
Correct VRE shophouse basis (land, not built units) and cut text ~46%
A prior draft argued the 2027 booking was safe because VRE "resells
finished stock" so handover follows sale within months. Wrong: the
Feb-2025 disclosures state the VND5,480bn deposit purchased COMMERCIAL
LAND PLOTS (109,800 sqm net floor, ~1,200 shophouses) from Vinhomes and
Vingroup - VRE develops them. Revenue books on handover, so a 2027
contribution needs construction complete by then, which is not
evidenced; the supporting claim that Royal Island construction finishes
in 2026 came only from property marketing sites, not an acceptable
source.

Growth cell now states the mechanism plainly instead of asserting a
booking case, and is cut from 1,504 to 819 characters. Internal record
carries the correction and notes leasing-only FY27F = 5,922 (+8.0%).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
+++ b/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
@@ -1296,7 +1296,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Deposit paid for shophouse land</t>
+          <t>Deposit — for LAND, not built units</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -1316,12 +1316,12 @@
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>MarketTimes; paid end-2024 for ~109,800 sqm net floor</t>
+          <t>MarketTimes / Nguoi Quan Sat, Feb-2025: VND5,480bn deposited end-2024 with Vinhomes/Vingroup for COMMERCIAL LAND PLOTS, 109,800 sqm net floor = ~1,200 shophouses</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>~1,200 units: Vinhomes Royal Island (~1,000) + Golden Avenue (~280).</t>
+          <t>CORRECTED. A draft claimed VRE resells "finished stock" so handover follows sale within months — WRONG. The deposit bought land; VRE develops. Revenue books on handover, so a 2027 contribution requires construction complete by then, which is not evidenced. Marketing-site claims that Royal Island construction completes in 2026 are NOT an acceptable source. Leasing-only FY27F would be 5,922 (+8.0%).</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="G35" s="12" t="inlineStr">
         <is>
-          <t>CORRECTED. An earlier draft said "management expects to contribute from 2027" — that was a journalist's passive phrasing, not a management statement, and it conflated SALES LAUNCH with REVENUE RECOGNITION. Booking case now rests on VRE reselling finished stock (units built out through 2026), so handover follows sale within months. Risk: sales opening late in 2027 pushes recognition to 2028.</t>
+          <t>CORRECTED. An earlier draft said "management expects to contribute from 2027" — that was a journalist's passive phrasing, not a management statement, and it conflated SALES LAUNCH with REVENUE RECOGNITION. Booking case is NOT established: VRE bought land and develops, so 2027 revenue depends on construction completing alongside the sales launch. Risk: sales opening late in 2027 pushes recognition to 2028.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add VPB HotStock package for the 31 Jul 2026 slot
- HotStock_VPB_31July2026.pptx: 4-slide Vietnamese deck in the BC mobile
  format (cover with BUY / TP 33,800, key-points panel, quarterly
  consolidated PBT chart 1Q25-2Q26, disclaimer appendix)
- HotStock_VPB_31July2026_script.md: 191-word broadcast script plus
  pre-recording checks
- INTERNAL_Sources_and_Assumptions_Aug26.xlsx: new "VPB HotStock" sheet
  recording the source of every figure, the derivation of the 3Q25/4Q25
  chart columns, and six known gaps

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
+++ b/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources &amp; Assumptions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VPB HotStock" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -475,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1771,21 +1772,6 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A3:G3"/>
@@ -1793,4 +1779,1164 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
+    <col width="68" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INTERNAL — NOT FOR DISTRIBUTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sources &amp; assumptions record — VPB HotStock, broadcast 31/07/2026 (Đạt Quân)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>RULE: no figure enters the deck or the script without a source. DERIVED = arithmetic on sourced figures, shown in full.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Source type</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Source detail / date</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Status &amp; notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>VPB — 1H26 REPORTED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>PBT 1H26 (consolidated)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>18,880</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY + PRESS</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>VPBank 1H26 release, 17/07/2026: "gần 18,900 tỷ, +68% CK, ~46% kế hoạch năm"</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Exact 18,880 = 1Q26 7,921 + 2Q26 10,959. The "+49%" figure seen earlier in the screen was a different scope and is dropped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>PBT 2Q26</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>10,959</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>PRESS</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Coverage of the 2Q26 consolidated FS: +76% YoY, highest in 4 years</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Cross-check: 18,880 − 7,921 = 10,959. Consistent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>PBT 1Q26</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>7,921</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY + PRESS</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>1Q26 release, 17/04/2026: "trên 7,900 tỷ, +58% CK"</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Exact value taken as 18,880 − 10,959.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>TOI 1H26</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>43,400 (+35.2%)</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>1H26 release; parent bank contributed &gt;31,600 (+35%)</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Parent figure is a contribution to TOI, not a profit figure — do not restate as profit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Total assets end-Jun-26</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>&gt;1,500,000 (+19.2% vs end-25)</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>1H26 release</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Credit balance, parent bank</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>~1,060,000 (+24.6% YTD)</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>1H26 release</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Parent-bank scope. Consolidated credit &gt;1,180,000 (+23% YTD) per the same release.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>NPL</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>parent ~2% (Circular 31); consolidated &lt;3%</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>1H26 release</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>TWO DIFFERENT SCOPES. Never quote one as the other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>VPB — BASE YEAR AND PLAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>FY25 PBT</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>30,600 (+53%)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>FY25 release, 19/01/2026; 121% of plan</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>Parent bank 26,300 (+44.4%). Subsidiaries FY25: VPBankS 4,476 (4x), OPES &gt;638, FE Credit &gt;600.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>9M25 PBT</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>20,400</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>9M25 release</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Rounded in the release ("hơn 20,400").</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>FY26 plan PBT</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>41,323 (+35%)</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>AGM 22/04/2026</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>VPB — DERIVED QUARTERLY SERIES (chart on slide 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>PBT 2Q25</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>6,230</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F19" s="7">
+        <f> 10,959 / 1.76 (2Q26 +76% YoY)</f>
+        <v/>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Implies 1H25 = 11,240; check 18,880 / 11,240 = +68.0% — matches the reported growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>PBT 1Q25</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>5,010</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F20" s="7">
+        <f> 7,921 / 1.58 (1Q26 +58% YoY)</f>
+        <v/>
+      </c>
+      <c r="G20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>PBT 3Q25</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>9,160</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F21" s="7">
+        <f> 20,400 (9M25) − 11,240 (1H25)</f>
+        <v/>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Cumulative sources are rounded, so this carries a few hundred bn of rounding error. Chart footnote says so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>PBT 4Q25</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>10,200</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F22" s="7">
+        <f> 30,600 (FY25) − 20,400 (9M25)</f>
+        <v/>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>Same rounding caveat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>PBT 2H25</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>~19,360</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F23" s="7">
+        <f> 30,600 − 11,240</f>
+        <v/>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>This is the base that makes 2H26 growth optics slow sharply — the main caveat in the script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>2H26 PBT needed to hit plan</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>22,443 (+16% YoY)</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F24" s="7">
+        <f> 41,323 − 18,880</f>
+        <v/>
+      </c>
+      <c r="G24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>VPB — CAPITAL INCREASE AND FOREIGN ROOM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Charter capital</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>79,339 → 106,243</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>AGM 22/04/2026</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Would be the largest in the system.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>Step 1 — stock dividend</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>26.04% (~2.06bn shares)</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Written consent: record date 30/06/2026, deadline 16/07/2026; execution expected 3Q–4Q26</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Source switched from capital surplus + reserve funds to &gt;20,660bn of retained earnings. NOT YET EXECUTED as at 30/07/2026 — the price and TP are both pre-dilution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Step 2 — private placement</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>624mn shares (~6,243bn)</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>shares</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY + PRESS</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>AGM 22/04/2026; expected 3Q–4Q26; foreign ownership could reach ~34%</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Buyer described as an existing strategic shareholder or a qualifying foreign institution — NOT NAMED. Do not name one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Decree 69/2025/NĐ-CP</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>foreign cap up to 49%</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>REGULATION</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Effective 19/05/2025; applies to banks receiving mandatory transfers of weak banks — VPB (GPBank), MBB (MBV), HDB (Vikki)</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Not automatic: needs a specific approval. Current foreign ownership: VPB 24.3%, MBB 22.3%, HDB 16.9%. Excludes banks &gt;50% state-owned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Cash dividend</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>5% of par (&gt;3,900bn)</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>COMPANY</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>FY25 dividend announcement</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>VPB — PRICE, TP, FORECAST</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Share price</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>24,600</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>VND/share</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>PRESS</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>Quoted for 28/07/2026; 24,950 on 24/07/2026</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>FROM A SEARCH SNIPPET, NOT A MARKET FEED (FiinQuant connector not authorised). Refresh before recording.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>MAS target price</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>33,800</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>VND/share</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Stock_Pick_and_Forecast_Aug26_MAS_RS_EN_updated.xlsx, Target Price sheet row 7</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Pre-dilution basis. After a 26.04% stock dividend this is ~26,800 — say "pre-dilution" if asked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Upside to TP</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>+37.4%</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F34" s="7">
+        <f> 33,800 / 24,600 − 1</f>
+        <v/>
+      </c>
+      <c r="G34" s="7" t="inlineStr">
+        <is>
+          <t>Moves with the price; recheck on the day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>MAS 2026F NPATMI</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>29,056</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Same file</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>MAS 2027F NPATMI</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>36,119 (+24.3%)</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Same file</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>KNOWN GAPS — read before recording</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>G1 FY25 NPATMI not sourced</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr"/>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>So the script quotes no 2026F NPATMI growth rate. Only the absolute 2026F/2027F figures and the 2027F growth are used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>G2 Forecast looks stale</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr"/>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>MAS 2026F NPATMI 29,056 implies PBT materially below the 41,323 plan, yet 1H26 is already at ~46% of plan and 2Q26 set a record. The VPB model looks due for an upgrade; not revised for this HotStock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>G3 No NPL chart</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr"/>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr"/>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Quarterly NPL bucket data for VPB was not obtained, so the deck has one chart instead of the two in the STB/EIB mobile reports. Spec allows 1–2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>G4 TP predates 2Q26</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr"/>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>TP 33,800 was set before the 2Q26 print and has not been re-derived here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>G5 Derived quarters</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr"/>
+      <c r="G42" s="7" t="inlineStr">
+        <is>
+          <t>3Q25 and 4Q25 chart columns are arithmetic on rounded cumulative disclosures — footnoted on the slide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>G6 No visual QA</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr"/>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>LibreOffice cannot open .pptx in this environment, so slide layout was verified by XML/text inspection only. Open the deck once before recording — SmartArt text is longer than the template original and PowerPoint will re-fit it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
VPB HotStock: 5-slide deck and Word version of the script
- Deck goes to 5 slides: adds a half-year PBT chart (1H25, 2H25, 1H26, and
  the 22,443bn 2H26 needs to hit the 41,323bn plan) so the high 2H25 base
  is visible rather than only mentioned. Both charts now use explicit
  srgbClr fills instead of a themeOverride part.
- Adds HotStock_VPB_31July2026_script.docx: the broadcast script as a Word
  document with a header block, the 191-word text, the slide list and the
  pre-recording checks.
- Internal sheet: records the slide-4 derivations and flags that the
  22,443bn column is a plan requirement, not a MAS forecast.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
+++ b/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
@@ -2382,7 +2382,7 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>This is the base that makes 2H26 growth optics slow sharply — the main caveat in the script.</t>
+          <t>Base for the 2H26 slowdown point. Plotted on slide 4 alongside 1H25 = 11,240 (= 18,880 / 1.68), 1H26 = 18,880 and the 22,443 needed for plan.</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,11 @@
         <f> 41,323 − 18,880</f>
         <v/>
       </c>
-      <c r="G24" s="7" t="inlineStr"/>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>Plotted as the 4th column of the slide-4 chart in a lighter colour and labelled "2H26 cần để đạt KH". IT IS NOT A MAS FORECAST — slide footnote says so explicitly.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
@@ -2851,7 +2855,7 @@
       <c r="F40" s="7" t="inlineStr"/>
       <c r="G40" s="7" t="inlineStr">
         <is>
-          <t>Quarterly NPL bucket data for VPB was not obtained, so the deck has one chart instead of the two in the STB/EIB mobile reports. Spec allows 1–2.</t>
+          <t>Quarterly NPL bucket data for VPB was not obtained, so the deck carries two PBT charts (quarterly and half-yearly) instead of the profit + NPL pair used in the STB/EIB mobile reports. Spec allows 1-2 visuals.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cut the FPT AI section to 100 words
The previous expansion ran long. The AI section is now 100 words in English
(125 in Vietnamese, which counts higher for the same text because the language
is monosyllabic), covering only the debate itself: the sector question, Infosys
at 8.2% AI revenue yet guiding FY27 to 1.5-3.0%, TCS growing 3.2% while adding
a net 9,279 staff, and FPT's Global IT at +13.4%.

The Global IT outlook that had been folded into the AI section — +16.7% FY27F,
Japan +22%/+23%, EU +18%/+20% and the US cut to +5.9% — moves back to the
segment paragraph where it belongs. No figure is lost.

Net effect on page length is -2.0% English and -3.1% Vietnamese against the
version before the expansion: the AI debate takes the space that the price
commentary and the deal list used to occupy. STB pages unchanged; all
arithmetic and parity checks pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
+++ b/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
@@ -3392,7 +3392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5185,6 +5185,81 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr"/>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Độ dài đoạn AI (sửa lần 2)</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>EN 100 từ / VN 125 từ</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr"/>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr"/>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>Yêu cầu 50-100 từ. Tiếng Việt đơn âm nên cùng một nội dung đếm ra nhiều từ hơn khoảng 25%; đây là bản dịch sát của đoạn tiếng Anh 100 từ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr"/>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Tổng độ dài trang FPT</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>EN -2.0% / VN -3.1% so với bản trước</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr"/>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr"/>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>Không còn tăng +15% như lượt trước. Đoạn AI thay chỗ cho phần mô tả diễn biến giá và danh sách hợp đồng, nên trang gần như giữ nguyên độ dài.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr"/>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Chi tiết CNTT nước ngoài</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>chuyển từ đoạn AI sang đoạn phân khúc</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr"/>
+      <c r="E73" s="6" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr"/>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>+16.7% FY27F, Nhật +22%/+23%, châu Âu +18%/+20%, Mỹ +5.9% nay nằm ở đoạn 2 để đoạn AI chỉ còn phần tranh luận. Không mất số nào.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
STB: fix FY26F PBT at VND8,150bn
Model!Y278 specific charge / write-off ratio 0.85x -> 0.8802x. Provisioning
11,091 -> 11,447 (+0.6% YoY), PBT 8,150 (+6.9% YoY, 0.6% above the ~8,100bn
board plan), NPATMI 6,346. Coverage 50.0% -> 51.0%. NPL 5.5% and the 40/38/36%
CIR path are untouched, as are FY27F and FY28F PBT at 14,676 and 21,145.

Also caught a rounding inconsistency while cascading: the narrative carried
+6.8% YoY where the summary box computed +6.9% from the same PBT. check_stb.py
now asserts the narrative's growth figure against the box, so the two cannot
drift apart again.

Deck, stock-pick workbook, Word note and audit trail updated. 107/107 pass.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
+++ b/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
@@ -3397,7 +3397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G235"/>
+  <dimension ref="A1:G260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9895,6 +9895,824 @@
         </is>
       </c>
       <c r="G235" t="inlineStr">
+        <is>
+          <t>Toàn bộ số ở trên tính lại bằng Python theo đúng chuỗi công thức của model (fix_stb_model.cascade); cần mở Excel đối chiếu trước khi phát hành</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="B237" s="13" t="inlineStr">
+        <is>
+          <t>STB — REVISION 04/08/2026: giữ bao phủ 50% -&gt; NPL 5.5%; CIR 40/38/36% FY26-28F</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Dự phòng đã trích cuối Q2/2026</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>27,177</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>MODEL</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>FinModel_STB_2Q26 Model!CA cột quý 2Q26; FY25 20,056 + 7,119 trích 1H26</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>Bao phủ 56.7% (27,177/47,957), tăng từ 50.0% cuối 2025 — gần như chưa xóa nợ trong 1H26</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Xóa nợ FY26F</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>11796</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>Model!Y287 = -1.71% x dư nợ 689,832 (trước: -0.95%)</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>Nghiệm của bài toán giữ bao phủ 50%; tương đương 37% dư nợ nhóm 5 (~32,000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Tỷ lệ trích/xóa FY26F</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>0.8802x</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>Model!Y278 = -Y279*0.8802 (1.5x -&gt; 0.85x -&gt; 0.8802x)</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Xử lý nợ tài trợ từ nguồn dự phòng đã trích, không từ P&amp;L. Giữ 1.5x trên mức xóa nợ này là nguyên nhân làm LNTT sụt 64% mà CV đã bác</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Dự phòng đã trích cuối FY26F / bao phủ</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>19330 / 50.9%</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>VNDbn / %</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>gen 4,665 + spec 14,309; NPL 5.5% x 689,832 = 37,941</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Đúng mục tiêu "giữ bao phủ 50%" của CV</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>R5</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>NPL FY26F / FY27F / FY28F</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>5.5 / 4.0 / 2.7</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>NPL!N26=0.933 N27=0.012 N28=0.009 N29=0.012 N30=0.034 (tổng 1.000)</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>Hàm ý nợ xấu phát sinh mới 2H26 = 1,780 tỷ, bằng 23% nhịp 1H26 (7,800) — khớp giả định "chậm lại còn 20% nhịp 1H" CV đưa ra trước đó</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>R6</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>CIR FY26F / FY27F / FY28F</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>40.0 / 38.0 / 36.0</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>Model!Y132=X132*1 và Y134=X134*1 (lương và chi phí khác đi ngang so với FY25); Z132/Z134 = *1.015; AA132/AA134 = *1.106. Khấu hao Y133/Z133/AA133 giữ nguyên build cũ</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>CIR 1H26 thực tế 35.6% (opex 6,233 / TOI 17,488). Build cũ cho 42.9/42.6/40.5%, tức opex 2H26 phải tăng 26.7% so với 1H26 — không có cơ sở. Hệ số nhân là nghiệm của mục tiêu CIR CV đặt ra, áp chung cho cả dòng lương và chi phí khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>R6b</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Ràng buộc của mục tiêu CIR 38% năm FY27F</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>+1.5%</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>% tăng opex</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>TOI FY27F +11.1% nhưng khấu hao Z133 = Y133*1.2 (+20%) theo build gốc</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Khấu hao nhảy 20% chiếm hết dư địa, nên lương + chi phí khác chỉ được tăng 1.5% để về 38%. Nếu hệ số khấu hao 1.2x không có cơ sở (đây là input của bản gốc, tôi không sửa), hạ về 1.1x sẽ cho lương + chi phí khác tăng 4.3% — hợp lý hơn. CẦN CV XÁC NHẬN</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Opex 2H26 hàm ý</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>6831</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>FY26F 13065 - 1H26 thực tế 6,233</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>+9.6% so với 1H26 — vẫn phản ánh tính mùa vụ dồn về cuối năm, không phải cắt giảm chi phí</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>R8</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>LNTT / LNST FY26F</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>8151 / 6346</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>TOI 32,956 - opex 13065 - dự phòng 11447</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>+6.9% CK. Hàm ý LNTT 2H26 4015 tỷ = 14x nền 2H25 (297 tỷ) và +-2.9% so với 1H26</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>R9</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Dự phòng P&amp;L FY26F</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>11447</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>chung 687 + cụ thể 10,027 + VAMC 377</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>-2.6% CK so với 11,384 của FY25; gần như không đổi so với 10,889 của bản trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Model!X284 dự phòng cụ thể đầu kỳ</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>4,891 -&gt; 16,078</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Model!X264 (BCĐKT FY25) = 20,056 nhưng bảng chuyển động X274+X284 chỉ 8,869</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>Lỗi có sẵn trong model: mọi tỷ lệ bao phủ dự phóng trước đây đều vô nghĩa. Đã sửa để X274+X284 = 20,056</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Cân đối kế toán sau khi sửa X284</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>MODEL</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>Model!Y103 = 0 sau khi CV mở lại bằng Excel (bản 2b63c432)</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>ĐÃ ĐÓNG — cảnh báo lệch -6,755 tỷ của tôi là SAI. Model tự cân đối; tổng tài sản Y61 = 1,014,277 (không phải 1,007,118 tôi ước tính)</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Đối chiếu sau khi Excel tính lại</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>khớp</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>MODEL</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>bản 2b63c432 do CV mở lại bằng Excel</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>Opex Y135 13,182/13,913/15,367 khớp tuyệt đối; dự phòng Y254 11,091 khớp; dự phòng đã trích Y286 18,973 và bao phủ 50.0% khớp tuyệt đối</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>TOI dịch chuyển khi Excel tính lại</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>32,662 vs 32,956</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>Model!Y117 = NII + phí + thu nhập khác</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>Dự phòng đã trích lớn hơn làm cho vay thuần giảm -&gt; thu nhập lãi giảm. NII FY26F về 26,712 (+0.1% CK) từ 27,010. Hệ quả CIR trôi lên 40.36/37.66/36.48%, đã giải lại hệ số nhân opex về 0.9886/1.039/1.0739 để đúng 40/38/36%</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>NPL!DG6:DG11 cột 2Q26</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>BY -&gt; BX</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>trỏ sang 'Notes(Quarter)'!BX81:BX86 (cột chèn thêm đẩy dữ liệu sang BX, BW là cột nhãn)</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>Tổng 636,029; nhóm 1-5: 571,245 / 16,827 / 7,200 / 8,483 / 32,274. NPL 47,957 = 7.540% — khớp tuyệt đối con số trên slide</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>G19</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>NPL hàng 19-21 lệch một dòng ở khối theo quý</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>DF19 = DF8/DF$22 (nợ nhóm 2 / nợ xấu) trong khi nhãn ghi "3) Substandard"</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>CHƯA SỬA — lỗi có sẵn ở MỌI cột quý, không riêng 2Q26; hàng 19-21 cộng lại không bằng 100%. Không ảnh hưởng tỷ lệ NPL (hàng 23) vì hàng 22 = SUM(9:11) vẫn đúng. Sửa riêng cột DG sẽ phá nhóm shared formula</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Giá mục tiêu vs sheet Valuation</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>77,800 vs 65,600</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>Valuation!B1 = J16 = P/B hợp lý FY27F x BPS FY27F</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Sheet Valuation cho 56,100 trước điều chỉnh và ~65,600 sau (ROE bền vững FY27F lên 15.5%, BPS 37,822). Slide vẫn để 77,800 — CHƯA ĐỊNH GIÁ LẠI, cần CV quyết</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>G16</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Giá mục tiêu ghi 77,500 trong file stock pick</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>77,500 vs 77,800</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>Stock Pick!D6 và Target Price!C13 ghi 77,500; cột J6/L6 lại tính trên 77,800</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>CHƯA SỬA — chênh 0.4%, cần CV xác nhận số nào đúng</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>LNTT FY26F chốt cứng</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>8,150</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>Model!Y278 = 0.8802x; dự phòng 11,091 -&gt; 11,447 (+0.6% CK)</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>CV chốt 8,150 tỷ (+6.9% CK, nhỉnh hơn kế hoạch 8,100 0.6%). Phần chênh lấy từ chi phí dự phòng, không đụng NPL 5.5% hay CIR 40%. Bao phủ 50.0% -&gt; 51.0%. Các bản trung gian đã thử 8,100 (0.8845x) và 8,507 = KH +5% (0.85x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Kế hoạch LNTT FY26 8,100 tỷ</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>suy ra</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>Suy ra từ 4,136/51% theo trích dẫn báo chí "hoàn thành 51% mục tiêu"</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>CHƯA CÓ NGHỊ QUYẾT ĐHĐCĐ TRONG HỒ SƠ. Nay con số này là mỏ neo của dự phóng LNTT nên cần lấy nguồn gốc trước khi phát hành. KH FY25 ~14,670 (7,628/52%) cũng suy ra tương tự</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Slide ghi "ban lãnh đạo dự kiến ~5.6%" nợ xấu</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>5.6%</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>Dòng 10 ghi 5.6% xuất hiện ở bản 24/07 dưới dạng "ước ~5.6%" — tức ước tính của MAS</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>CHƯA SỬA — slide đang gán cho ban lãnh đạo. Nếu không có công bố của STB thì phải viết lại, đây là chỗ duy nhất trong khối STB có nguy cơ trình bày ước tính MAS như guidance</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>G17</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Tăng trưởng tín dụng FY26F 11.7% vs 1.5% thực hiện 1H26</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Model!Y206 = 10.1%; slide ghi 11.7%</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>CHƯA XỬ LÝ — CV đã cân nhắc dùng làm đòn bẩy đưa LNTT về kế hoạch nhưng chọn dự phòng. Dư nợ dựng từ dưới lên theo 6 phân khúc (Model!Y23:Y28) nên phải tính lại bằng Excel</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>G18</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Model chưa mở lại bằng Excel</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>fullCalcOnLoad=1 đã bật</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
         <is>
           <t>Toàn bộ số ở trên tính lại bằng Python theo đúng chuỗi công thức của model (fix_stb_model.cascade); cần mở Excel đối chiếu trước khi phát hành</t>
         </is>

</xml_diff>

<commit_message>
STB: FY28F PBT down a further VND1,000bn
The FY28F provisioning overlay goes from VND1,000bn to VND2,000bn
(Model!AA278 = -AA279+2000), taking PBT to VND15,271bn.

Booked on the provisioning line rather than the income lines because CIR is
pinned at 42.1 / 40 / 38%: cutting TOI would have forced a matching opex cut to
hold the ratio, i.e. two levers for one outcome.

  Provisioning  10,202 / 10,636 /  8,982
  PBT            7,461 /  9,872 / 15,271  (FY28F was 16,271)
  NPATMI         5,809 /  7,686 / 11,890
  ROE              8.8 /   11.0 /   15.0%
  P/E @75,000     26.6 /   20.1 /   13.0

FY28F growth lands at +54.7%, close to the 50% set in the challenge round.
NPL coverage reaches 105% by FY28F against 91% before either tranche - logged
as G22 with the alternative lever, the unexplained 1.7x uplift on FY28F
recovery income, logged as G23.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPsxWfyBSmSQjUzo5EDnm5
</commit_message>
<xml_diff>
--- a/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
+++ b/INTERNAL_Sources_and_Assumptions_Aug26.xlsx
@@ -3397,7 +3397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G288"/>
+  <dimension ref="A1:G299"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11570,6 +11570,326 @@
         </is>
       </c>
       <c r="G288" t="inlineStr">
+        <is>
+          <t>ROE FY27F nay chỉ còn 11.0% nên P/B hợp lý tính lại còn thấp hơn nữa. CHƯA ĐỊNH GIÁ LẠI</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="B290" s="13" t="inlineStr">
+        <is>
+          <t>STB — REVISION 05/08/2026 b (dự phòng FY27F +1,000, FY28F +2,000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Trích thêm dự phòng FY27F và FY28F</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>1,000 / 2,000</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>MAS</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Model!Z278 = -Z279+1000, AA278 = -AA279+2000 (trước đó = -Z279*1, -AA279*1)</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Viết dạng cộng thẳng thay vì hệ số nhân để phần trích thêm hiện rõ trong ô. Tỷ lệ xóa nợ -1.2%/-0.7% giữ nguyên nên phần trích thêm không dùng để xóa nợ mà bồi đắp bộ đệm: dự phòng đã trích tăng 1,000 tỷ năm FY27F và 3,000 tỷ lũy kế FY28F. Đợt 2,000 tỷ ở FY28F là yêu cầu hạ LNTT FY28F thêm 1,000 tỷ — dùng cùng một đòn bẩy để CIR 38% và các dòng thu nhập giữ nguyên</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>A9</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Chi phí dự phòng FY26F / FY27F / FY28F</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>10202 / 10636 / 8982</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>MODEL</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Model!Y/Z/AA141</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>FY27F từ 9,636 lên 10,636; FY28F từ 6,982 lên 8,982</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>LNTT FY27F / FY28F</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>9872 / 15271</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>MODEL</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Model!Z144 / AA144</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>FY27F từ 10,872 xuống 9872 (+32.3% CK, trước là +45.7%); FY28F từ 17,271 xuống 15271 (+54.7% CK, trước là +58.9%) — sát mục tiêu 50% CV đặt ở vòng trước</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>LNST / ROE FY27F / FY28F</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>7686 / 11890</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>VNDbn</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>MODEL</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Model!Z153, AA153, Z314, AA314</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>ROE FY27F 11.0% (từ 12.1%), FY28F 15.0% (từ 16.6%). Vốn chủ cuối FY28F 85305 tỷ, thấp hơn 2,336 tỷ so với bản trước do lợi nhuận giữ lại giảm</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>A12</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>P/E, P/B FY27F / FY28F trên giá mục tiêu 75,000</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>20.1 / 13.0 x</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>DERIVED</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>EPS FY27F 3731, FY28F 5771 trên 2060 triệu cổ phiếu</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>P/E FY27F từ 18.3 lên 20.1, FY28F từ 11.5 lên 13.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>G21</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Đỉnh dự phòng dời từ FY26F sang FY27F</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Dự phòng 10202 / 10636 / 8982 trong khi xóa nợ 10,955 / 8,637 / 5,779</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Phần trích thêm đẩy chi phí FY27F vượt FY26F dù xóa nợ giảm 21%. Đây là hệ quả trực tiếp của yêu cầu, không phải lỗi, nhưng làm chậm câu chuyện hồi phục một năm</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>G22</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Bao phủ nợ xấu FY28F chạm ~100%</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>51 / 71 / 105%</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Dự phòng đã trích 18926 / 20524 / 23305 trên nợ xấu 37157 / 28791 / 22290</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Trước khi trích thêm là 50.9 / 67.8 / 91.1%. Bao phủ trên 100% ở một ngân hàng vừa xử lý xong tồn đọng là mức của nhóm đầu ngành — CV cân nhắc có muốn giữ hay chuyển phần hạ LNTT FY28F sang dòng thu nhập (xem G23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>G23</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Đòn bẩy thay thế: hệ số 1.7x ở thu nhập khác FY28F</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>GAP</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Model!AA129 = Z129/Z130*AA130*1.7 — thu hồi nợ đã xóa tăng 34% trong khi xóa nợ giảm 33% (8,637 -&gt; 5,779)</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>CHƯA SỬA. Bỏ hệ số 1.7 sẽ hạ thu nhập khác FY28F 1,123 tỷ, tức cũng đạt mục tiêu hạ LNTT, nhưng kéo CIR FY28F từ 38.0% lên 39.1% nên phải giải lại hệ số chi phí</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Giá mục tiêu STB vs sheet Valuation</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>75,000 vs ~46,500</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>CONFLICT</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Valuation: P/B hợp lý (ROE 12.1% - 2.5%) / (10.01% - 2.5%) = 1.29x x BPS 36,014</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
         <is>
           <t>ROE FY27F nay chỉ còn 11.0% nên P/B hợp lý tính lại còn thấp hơn nữa. CHƯA ĐỊNH GIÁ LẠI</t>
         </is>

</xml_diff>